<commit_message>
need to edit Site names in spreadsheet to match sites_stratav7
</commit_message>
<xml_diff>
--- a/survey_wqdata/SR_Data_editsv1.xlsx
+++ b/survey_wqdata/SR_Data_editsv1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\atweg\Documents\Mike\Nokuse\R_sevensrun\nokuse_seven_runs_survey\survey_wqdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1EE46D0B-F9B5-47D5-97F2-C8BC9F031559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{906FD5AB-B4CA-4A53-B2EC-FBA49A47FBE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{BC263282-6D8F-47C7-8BF3-A88688F790FA}"/>
   </bookViews>
@@ -23,17 +23,6 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -42,24 +31,6 @@
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="66">
   <si>
     <t>Site</t>
-  </si>
-  <si>
-    <t>sr_mst_a</t>
-  </si>
-  <si>
-    <t>sr_mst_b</t>
-  </si>
-  <si>
-    <t>sr_mst_c</t>
-  </si>
-  <si>
-    <t>sr_mst_d</t>
-  </si>
-  <si>
-    <t>sr_mst_e</t>
-  </si>
-  <si>
-    <t>sr_mst_f</t>
   </si>
   <si>
     <t>mck_br_a</t>
@@ -270,13 +241,31 @@
   <si>
     <t>Dip net x10: crayfish, Gambusia, dragonfly larvae</t>
   </si>
+  <si>
+    <t>mst_a</t>
+  </si>
+  <si>
+    <t>mst_b</t>
+  </si>
+  <si>
+    <t>mst_c</t>
+  </si>
+  <si>
+    <t>mst_d</t>
+  </si>
+  <si>
+    <t>mst_e</t>
+  </si>
+  <si>
+    <t>mst_f</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -332,8 +321,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
@@ -695,93 +684,93 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I1" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="J1" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="K1" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="L1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="M1" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="H1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="O1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="P1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="R1" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="S1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="L1" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="M1" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="N1" s="5" t="s">
+      <c r="T1" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="U1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="V1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="X1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="Q1" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="R1" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="S1" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="T1" s="5" t="s">
+      <c r="Y1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="W1" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>46</v>
-      </c>
       <c r="AB1" s="1" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:28">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="B2" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C2" s="2">
         <v>45909</v>
@@ -796,7 +785,7 @@
         <v>-86.038640000000001</v>
       </c>
       <c r="G2" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H2" s="6">
         <v>0.25</v>
@@ -823,7 +812,7 @@
         <v>1.63</v>
       </c>
       <c r="P2" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="Q2" s="6">
         <v>1.37</v>
@@ -838,42 +827,42 @@
         <v>99.48</v>
       </c>
       <c r="U2" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="V2" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="W2" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="X2" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="Y2" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="Z2" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="AA2" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="AB2" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:28">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>61</v>
       </c>
       <c r="B3" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C3" s="2">
         <v>45909</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="E3">
         <v>30.574836999999999</v>
@@ -882,7 +871,7 @@
         <v>-86.028282000000004</v>
       </c>
       <c r="G3" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H3" s="6">
         <v>0.38</v>
@@ -909,7 +898,7 @@
         <v>2.56</v>
       </c>
       <c r="P3" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="Q3" s="6">
         <v>2.69</v>
@@ -924,33 +913,33 @@
         <v>95.84</v>
       </c>
       <c r="U3" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="V3" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="W3" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="X3" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="Y3" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="Z3" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="AA3" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:28">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>62</v>
       </c>
       <c r="B4" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C4" s="2">
         <v>45909</v>
@@ -965,7 +954,7 @@
         <v>-86.016197000000005</v>
       </c>
       <c r="G4" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H4" s="6">
         <v>0.4</v>
@@ -992,7 +981,7 @@
         <v>2.14</v>
       </c>
       <c r="P4" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="Q4" s="6">
         <v>4.83</v>
@@ -1007,36 +996,36 @@
         <v>99.48</v>
       </c>
       <c r="U4" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="V4" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="W4" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="X4" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="Y4" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="Z4" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="AA4" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="AB4" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:28">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>63</v>
       </c>
       <c r="B5" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C5" s="2">
         <v>45912</v>
@@ -1051,7 +1040,7 @@
         <v>-85.978043</v>
       </c>
       <c r="G5" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H5" s="6">
         <v>0.32</v>
@@ -1078,7 +1067,7 @@
         <v>2.5099999999999998</v>
       </c>
       <c r="P5" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="Q5" s="6">
         <v>6.45</v>
@@ -1093,39 +1082,39 @@
         <v>84.92</v>
       </c>
       <c r="U5" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="V5" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="W5" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="X5" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="Y5" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="Z5" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="AA5" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:28">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>64</v>
       </c>
       <c r="B6" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C6" s="2">
         <v>45911</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="E6">
         <v>30.556989999999999</v>
@@ -1134,7 +1123,7 @@
         <v>-85.963539999999995</v>
       </c>
       <c r="G6" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H6" s="6">
         <v>0.32</v>
@@ -1161,7 +1150,7 @@
         <v>3.71</v>
       </c>
       <c r="P6" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="Q6" s="6">
         <v>5.13</v>
@@ -1176,33 +1165,33 @@
         <v>96.1</v>
       </c>
       <c r="U6" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="V6" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="W6" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="X6" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="Y6" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="Z6" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="AA6" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:28">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>65</v>
       </c>
       <c r="B7" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C7" s="2">
         <v>45911</v>
@@ -1217,7 +1206,7 @@
         <v>-85.962569000000002</v>
       </c>
       <c r="G7" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H7" s="6">
         <v>0.43</v>
@@ -1244,7 +1233,7 @@
         <v>2.33</v>
       </c>
       <c r="P7" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="Q7" s="6">
         <v>4.83</v>
@@ -1259,33 +1248,33 @@
         <v>92.72</v>
       </c>
       <c r="U7" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="V7" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="W7" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="X7" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="Y7" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="Z7" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="AA7" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:28">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C8" s="2">
         <v>45910</v>
@@ -1300,7 +1289,7 @@
         <v>-85.979294999999993</v>
       </c>
       <c r="G8" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H8" s="6">
         <v>0.32</v>
@@ -1327,7 +1316,7 @@
         <v>1.44</v>
       </c>
       <c r="P8" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="Q8" s="6">
         <v>1.65</v>
@@ -1342,33 +1331,33 @@
         <v>97.92</v>
       </c>
       <c r="U8" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="V8" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="W8" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="X8" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="Y8" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="Z8" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="AA8" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:28">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C9" s="2">
         <v>45910</v>
@@ -1383,7 +1372,7 @@
         <v>-85.980097000000001</v>
       </c>
       <c r="G9" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H9" s="6">
         <v>0.25</v>
@@ -1410,7 +1399,7 @@
         <v>1.74</v>
       </c>
       <c r="P9" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="Q9" s="6">
         <v>1.0900000000000001</v>
@@ -1425,33 +1414,33 @@
         <v>100</v>
       </c>
       <c r="U9" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="V9" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="W9" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="X9" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="Y9" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="Z9" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="AA9" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10" spans="1:28">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C10" s="2">
         <v>45910</v>
@@ -1466,7 +1455,7 @@
         <v>-85.979523</v>
       </c>
       <c r="G10" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H10" s="6">
         <v>0.25</v>
@@ -1493,7 +1482,7 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="P10" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="Q10" s="6">
         <v>2.82</v>
@@ -1508,42 +1497,42 @@
         <v>98.18</v>
       </c>
       <c r="U10" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="V10" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="W10" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="X10" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="Y10" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="Z10" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="AA10" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="AB10" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:28">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C11" s="2">
         <v>45910</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="E11">
         <v>30.567005999999999</v>
@@ -1553,7 +1542,7 @@
         <v>-85.979297000000003</v>
       </c>
       <c r="G11" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H11" s="6">
         <v>0.34</v>
@@ -1580,7 +1569,7 @@
         <v>3.08</v>
       </c>
       <c r="P11" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="Q11" s="6">
         <v>2.11</v>
@@ -1595,36 +1584,36 @@
         <v>98.44</v>
       </c>
       <c r="U11" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="V11" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="W11" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="X11" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="Y11" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="Z11" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="AA11" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="AB11" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12" spans="1:28">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B12" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C12" s="2">
         <v>45910</v>
@@ -1639,7 +1628,7 @@
         <v>-85.964935999999994</v>
       </c>
       <c r="G12" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H12" s="6">
         <v>0.23</v>
@@ -1666,7 +1655,7 @@
         <v>2</v>
       </c>
       <c r="P12" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="Q12" s="6">
         <v>1.4</v>
@@ -1681,33 +1670,33 @@
         <v>99.22</v>
       </c>
       <c r="U12" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="V12" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="W12" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="X12" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="Y12" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="Z12" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="AA12" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:28">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B13" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C13" s="2">
         <v>45910</v>
@@ -1722,7 +1711,7 @@
         <v>-85.966836999999998</v>
       </c>
       <c r="G13" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H13" s="6">
         <v>0.31</v>
@@ -1749,7 +1738,7 @@
         <v>2.48</v>
       </c>
       <c r="P13" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="Q13" s="6">
         <v>2.74</v>
@@ -1764,33 +1753,33 @@
         <v>99.48</v>
       </c>
       <c r="U13" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="V13" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="W13" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="X13" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="Y13" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="Z13" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="AA13" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" spans="1:28">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="B14" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C14" s="2">
         <v>45911</v>
@@ -1805,7 +1794,7 @@
         <v>-85.966802999999999</v>
       </c>
       <c r="G14" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H14" s="6">
         <v>0.3</v>
@@ -1832,7 +1821,7 @@
         <v>1.85</v>
       </c>
       <c r="P14" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="Q14" s="6">
         <v>2.62</v>
@@ -1847,33 +1836,33 @@
         <v>97.66</v>
       </c>
       <c r="U14" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="V14" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="W14" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="X14" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="Y14" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="Z14" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="AA14" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:28">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B15" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C15" s="2">
         <v>45912</v>
@@ -1885,78 +1874,78 @@
         <v>-85.984607999999994</v>
       </c>
       <c r="G15" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="L15" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="M15" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="N15" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="O15" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="P15" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="Q15" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="R15" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="S15" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="T15" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="U15" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="V15" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="W15" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="X15" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="Y15" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="Z15" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="AA15" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="AB15" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:28">
       <c r="A16" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B16" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C16" s="2">
         <v>45912</v>
@@ -1971,7 +1960,7 @@
         <v>-85.981594000000001</v>
       </c>
       <c r="G16" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H16" s="6">
         <v>0.22</v>
@@ -1998,7 +1987,7 @@
         <v>3.51</v>
       </c>
       <c r="P16" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="Q16" s="6">
         <v>2.72</v>
@@ -2013,33 +2002,33 @@
         <v>98.18</v>
       </c>
       <c r="U16" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="V16" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="W16" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="X16" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="Y16" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="Z16" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="AA16" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17" spans="1:28">
       <c r="A17" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B17" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C17" s="2">
         <v>45911</v>
@@ -2054,78 +2043,78 @@
         <v>-85.919370000000001</v>
       </c>
       <c r="G17" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="L17" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="M17" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="N17" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="O17" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="P17" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="Q17" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="R17" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="S17" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="T17" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="U17" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="V17" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="W17" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="X17" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="Y17" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="Z17" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="AA17" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="AB17" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:28">
       <c r="A18" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="B18" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C18" s="2">
         <v>45909</v>
@@ -2140,7 +2129,7 @@
         <v>-85.999088</v>
       </c>
       <c r="G18" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H18" s="6">
         <v>0.36</v>
@@ -2167,7 +2156,7 @@
         <v>2.82</v>
       </c>
       <c r="P18" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="Q18" s="6">
         <v>2.62</v>
@@ -2182,36 +2171,36 @@
         <v>99.74</v>
       </c>
       <c r="U18" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="V18" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="W18" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="X18" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="Y18" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="Z18" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="AA18" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="AB18" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
     </row>
     <row r="19" spans="1:28">
       <c r="A19" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="B19" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C19" s="2">
         <v>45911</v>
@@ -2226,7 +2215,7 @@
         <v>-85.935445999999999</v>
       </c>
       <c r="G19" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H19" s="6">
         <v>0.3</v>
@@ -2253,7 +2242,7 @@
         <v>3.1</v>
       </c>
       <c r="P19" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="Q19" s="6">
         <v>2.62</v>
@@ -2268,33 +2257,33 @@
         <v>97.4</v>
       </c>
       <c r="U19" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="V19" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="W19" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="X19" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="Y19" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="Z19" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="AA19" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="20" spans="1:28">
       <c r="A20" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C20" s="2">
         <v>45911</v>
@@ -2306,78 +2295,78 @@
         <v>-85.971446999999998</v>
       </c>
       <c r="G20" t="s">
+        <v>45</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="I20" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="J20" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="K20" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="L20" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="M20" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="N20" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="O20" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="P20" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q20" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="R20" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="S20" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="T20" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="U20" t="s">
+        <v>48</v>
+      </c>
+      <c r="V20" t="s">
+        <v>48</v>
+      </c>
+      <c r="W20" t="s">
+        <v>48</v>
+      </c>
+      <c r="X20" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>48</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB20" t="s">
         <v>51</v>
-      </c>
-      <c r="H20" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="I20" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="J20" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="K20" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="L20" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="M20" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="N20" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="O20" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="P20" t="s">
-        <v>54</v>
-      </c>
-      <c r="Q20" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="R20" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="S20" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="T20" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="U20" t="s">
-        <v>54</v>
-      </c>
-      <c r="V20" t="s">
-        <v>54</v>
-      </c>
-      <c r="W20" t="s">
-        <v>54</v>
-      </c>
-      <c r="X20" t="s">
-        <v>54</v>
-      </c>
-      <c r="Y20" t="s">
-        <v>54</v>
-      </c>
-      <c r="Z20" t="s">
-        <v>54</v>
-      </c>
-      <c r="AA20" t="s">
-        <v>54</v>
-      </c>
-      <c r="AB20" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="21" spans="1:28">
       <c r="A21" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="B21" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C21" s="2">
         <v>45911</v>
@@ -2389,70 +2378,70 @@
         <v>-85.958196000000001</v>
       </c>
       <c r="G21" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="J21" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="K21" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="L21" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="M21" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="N21" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="O21" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="P21" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="Q21" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="R21" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="S21" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="T21" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="U21" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="V21" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="W21" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="X21" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="Y21" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="Z21" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="AA21" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="AB21" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
dropping units from pH to see if cont_analysis function will work on that name. getting error with `pH (SU)`
</commit_message>
<xml_diff>
--- a/survey_wqdata/SR_Data_editsv1.xlsx
+++ b/survey_wqdata/SR_Data_editsv1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\atweg\Documents\Mike\Nokuse\R_sevensrun\nokuse_seven_runs_survey\survey_wqdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{906FD5AB-B4CA-4A53-B2EC-FBA49A47FBE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B4359B0-8CAD-48D6-A092-F3E29111E965}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{BC263282-6D8F-47C7-8BF3-A88688F790FA}"/>
   </bookViews>
@@ -31,18 +31,6 @@
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="66">
   <si>
     <t>Site</t>
-  </si>
-  <si>
-    <t>mck_br_a</t>
-  </si>
-  <si>
-    <t>mck_br_b</t>
-  </si>
-  <si>
-    <t>mck_br_c</t>
-  </si>
-  <si>
-    <t>mck_br_d</t>
   </si>
   <si>
     <t>sm_br_a</t>
@@ -258,6 +246,18 @@
   </si>
   <si>
     <t>mst_f</t>
+  </si>
+  <si>
+    <t>mck_a</t>
+  </si>
+  <si>
+    <t>mck_b</t>
+  </si>
+  <si>
+    <t>mck_c</t>
+  </si>
+  <si>
+    <t>mck_d</t>
   </si>
 </sst>
 </file>
@@ -684,93 +684,93 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="I1" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="J1" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="K1" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="L1" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="H1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="J1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="O1" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q1" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="R1" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L1" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M1" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="O1" s="5" t="s">
+      <c r="S1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="T1" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="V1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="Q1" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="R1" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="S1" s="5" t="s">
+      <c r="W1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="T1" s="5" t="s">
+      <c r="X1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="U1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="V1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="Y1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>40</v>
-      </c>
       <c r="AB1" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:28">
       <c r="A2" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C2" s="2">
         <v>45909</v>
@@ -785,7 +785,7 @@
         <v>-86.038640000000001</v>
       </c>
       <c r="G2" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H2" s="6">
         <v>0.25</v>
@@ -812,7 +812,7 @@
         <v>1.63</v>
       </c>
       <c r="P2" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q2" s="6">
         <v>1.37</v>
@@ -827,42 +827,42 @@
         <v>99.48</v>
       </c>
       <c r="U2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="V2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="W2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="X2" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="Y2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="Z2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="AA2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="AB2" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:28">
       <c r="A3" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B3" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C3" s="2">
         <v>45909</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E3">
         <v>30.574836999999999</v>
@@ -871,7 +871,7 @@
         <v>-86.028282000000004</v>
       </c>
       <c r="G3" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H3" s="6">
         <v>0.38</v>
@@ -898,7 +898,7 @@
         <v>2.56</v>
       </c>
       <c r="P3" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q3" s="6">
         <v>2.69</v>
@@ -913,33 +913,33 @@
         <v>95.84</v>
       </c>
       <c r="U3" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="V3" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="W3" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="X3" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="Y3" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="Z3" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="AA3" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:28">
       <c r="A4" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B4" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C4" s="2">
         <v>45909</v>
@@ -954,7 +954,7 @@
         <v>-86.016197000000005</v>
       </c>
       <c r="G4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H4" s="6">
         <v>0.4</v>
@@ -981,7 +981,7 @@
         <v>2.14</v>
       </c>
       <c r="P4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q4" s="6">
         <v>4.83</v>
@@ -996,36 +996,36 @@
         <v>99.48</v>
       </c>
       <c r="U4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="V4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="W4" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="X4" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="Y4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="Z4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="AA4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="AB4" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:28">
       <c r="A5" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B5" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C5" s="2">
         <v>45912</v>
@@ -1040,7 +1040,7 @@
         <v>-85.978043</v>
       </c>
       <c r="G5" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H5" s="6">
         <v>0.32</v>
@@ -1067,7 +1067,7 @@
         <v>2.5099999999999998</v>
       </c>
       <c r="P5" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q5" s="6">
         <v>6.45</v>
@@ -1082,39 +1082,39 @@
         <v>84.92</v>
       </c>
       <c r="U5" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="V5" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="W5" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="X5" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="Y5" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="Z5" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="AA5" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:28">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B6" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C6" s="2">
         <v>45911</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E6">
         <v>30.556989999999999</v>
@@ -1123,7 +1123,7 @@
         <v>-85.963539999999995</v>
       </c>
       <c r="G6" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H6" s="6">
         <v>0.32</v>
@@ -1150,7 +1150,7 @@
         <v>3.71</v>
       </c>
       <c r="P6" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q6" s="6">
         <v>5.13</v>
@@ -1165,33 +1165,33 @@
         <v>96.1</v>
       </c>
       <c r="U6" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="V6" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="W6" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="X6" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="Y6" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="Z6" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="AA6" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:28">
       <c r="A7" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B7" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C7" s="2">
         <v>45911</v>
@@ -1206,7 +1206,7 @@
         <v>-85.962569000000002</v>
       </c>
       <c r="G7" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H7" s="6">
         <v>0.43</v>
@@ -1233,7 +1233,7 @@
         <v>2.33</v>
       </c>
       <c r="P7" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q7" s="6">
         <v>4.83</v>
@@ -1248,33 +1248,33 @@
         <v>92.72</v>
       </c>
       <c r="U7" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="V7" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="W7" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="X7" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="Y7" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="Z7" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="AA7" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:28">
       <c r="A8" t="s">
-        <v>1</v>
+        <v>62</v>
       </c>
       <c r="B8" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C8" s="2">
         <v>45910</v>
@@ -1289,7 +1289,7 @@
         <v>-85.979294999999993</v>
       </c>
       <c r="G8" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H8" s="6">
         <v>0.32</v>
@@ -1316,7 +1316,7 @@
         <v>1.44</v>
       </c>
       <c r="P8" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q8" s="6">
         <v>1.65</v>
@@ -1331,33 +1331,33 @@
         <v>97.92</v>
       </c>
       <c r="U8" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="V8" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="W8" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="X8" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="Y8" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="Z8" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="AA8" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:28">
       <c r="A9" t="s">
-        <v>2</v>
+        <v>63</v>
       </c>
       <c r="B9" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C9" s="2">
         <v>45910</v>
@@ -1372,7 +1372,7 @@
         <v>-85.980097000000001</v>
       </c>
       <c r="G9" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H9" s="6">
         <v>0.25</v>
@@ -1399,7 +1399,7 @@
         <v>1.74</v>
       </c>
       <c r="P9" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q9" s="6">
         <v>1.0900000000000001</v>
@@ -1414,33 +1414,33 @@
         <v>100</v>
       </c>
       <c r="U9" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="V9" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="W9" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="X9" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="Y9" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="Z9" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="AA9" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:28">
       <c r="A10" t="s">
-        <v>3</v>
+        <v>64</v>
       </c>
       <c r="B10" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C10" s="2">
         <v>45910</v>
@@ -1455,7 +1455,7 @@
         <v>-85.979523</v>
       </c>
       <c r="G10" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H10" s="6">
         <v>0.25</v>
@@ -1482,7 +1482,7 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="P10" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q10" s="6">
         <v>2.82</v>
@@ -1497,42 +1497,42 @@
         <v>98.18</v>
       </c>
       <c r="U10" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="V10" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="W10" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="X10" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="Y10" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="Z10" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="AA10" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="AB10" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:28">
       <c r="A11" t="s">
-        <v>4</v>
+        <v>65</v>
       </c>
       <c r="B11" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C11" s="2">
         <v>45910</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E11">
         <v>30.567005999999999</v>
@@ -1542,7 +1542,7 @@
         <v>-85.979297000000003</v>
       </c>
       <c r="G11" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H11" s="6">
         <v>0.34</v>
@@ -1569,7 +1569,7 @@
         <v>3.08</v>
       </c>
       <c r="P11" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q11" s="6">
         <v>2.11</v>
@@ -1584,36 +1584,36 @@
         <v>98.44</v>
       </c>
       <c r="U11" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="V11" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="W11" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="X11" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="Y11" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="Z11" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="AA11" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="AB11" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:28">
       <c r="A12" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B12" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C12" s="2">
         <v>45910</v>
@@ -1628,7 +1628,7 @@
         <v>-85.964935999999994</v>
       </c>
       <c r="G12" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H12" s="6">
         <v>0.23</v>
@@ -1655,7 +1655,7 @@
         <v>2</v>
       </c>
       <c r="P12" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q12" s="6">
         <v>1.4</v>
@@ -1670,33 +1670,33 @@
         <v>99.22</v>
       </c>
       <c r="U12" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="V12" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="W12" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="X12" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="Y12" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="Z12" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="AA12" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:28">
       <c r="A13" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="B13" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C13" s="2">
         <v>45910</v>
@@ -1711,7 +1711,7 @@
         <v>-85.966836999999998</v>
       </c>
       <c r="G13" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H13" s="6">
         <v>0.31</v>
@@ -1738,7 +1738,7 @@
         <v>2.48</v>
       </c>
       <c r="P13" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q13" s="6">
         <v>2.74</v>
@@ -1753,33 +1753,33 @@
         <v>99.48</v>
       </c>
       <c r="U13" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="V13" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="W13" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="X13" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="Y13" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="Z13" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="AA13" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" spans="1:28">
       <c r="A14" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B14" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C14" s="2">
         <v>45911</v>
@@ -1794,7 +1794,7 @@
         <v>-85.966802999999999</v>
       </c>
       <c r="G14" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H14" s="6">
         <v>0.3</v>
@@ -1821,7 +1821,7 @@
         <v>1.85</v>
       </c>
       <c r="P14" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q14" s="6">
         <v>2.62</v>
@@ -1836,33 +1836,33 @@
         <v>97.66</v>
       </c>
       <c r="U14" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="V14" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="W14" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="X14" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="Y14" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="Z14" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="AA14" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:28">
       <c r="A15" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C15" s="2">
         <v>45912</v>
@@ -1874,78 +1874,78 @@
         <v>-85.984607999999994</v>
       </c>
       <c r="G15" t="s">
+        <v>41</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="K15" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="L15" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="M15" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="N15" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="O15" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="P15" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q15" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="R15" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="S15" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="T15" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="U15" t="s">
+        <v>44</v>
+      </c>
+      <c r="V15" t="s">
+        <v>44</v>
+      </c>
+      <c r="W15" t="s">
+        <v>44</v>
+      </c>
+      <c r="X15" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y15" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>44</v>
+      </c>
+      <c r="AB15" t="s">
         <v>45</v>
-      </c>
-      <c r="H15" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="I15" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="J15" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="K15" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="L15" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="M15" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="N15" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="O15" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="P15" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q15" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="R15" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="S15" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="T15" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="U15" t="s">
-        <v>48</v>
-      </c>
-      <c r="V15" t="s">
-        <v>48</v>
-      </c>
-      <c r="W15" t="s">
-        <v>48</v>
-      </c>
-      <c r="X15" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y15" t="s">
-        <v>48</v>
-      </c>
-      <c r="Z15" t="s">
-        <v>48</v>
-      </c>
-      <c r="AA15" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB15" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:28">
       <c r="A16" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B16" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C16" s="2">
         <v>45912</v>
@@ -1960,7 +1960,7 @@
         <v>-85.981594000000001</v>
       </c>
       <c r="G16" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H16" s="6">
         <v>0.22</v>
@@ -1987,7 +1987,7 @@
         <v>3.51</v>
       </c>
       <c r="P16" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q16" s="6">
         <v>2.72</v>
@@ -2002,33 +2002,33 @@
         <v>98.18</v>
       </c>
       <c r="U16" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="V16" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="W16" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="X16" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="Y16" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="Z16" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="AA16" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17" spans="1:28">
       <c r="A17" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B17" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C17" s="2">
         <v>45911</v>
@@ -2043,78 +2043,78 @@
         <v>-85.919370000000001</v>
       </c>
       <c r="G17" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="L17" s="6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="M17" s="6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="N17" s="6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="O17" s="6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="P17" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="Q17" s="6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="R17" s="6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="S17" s="6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="T17" s="6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="U17" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="V17" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="W17" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="X17" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="Y17" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="Z17" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="AA17" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="AB17" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="18" spans="1:28">
       <c r="A18" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B18" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C18" s="2">
         <v>45909</v>
@@ -2129,7 +2129,7 @@
         <v>-85.999088</v>
       </c>
       <c r="G18" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H18" s="6">
         <v>0.36</v>
@@ -2156,7 +2156,7 @@
         <v>2.82</v>
       </c>
       <c r="P18" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q18" s="6">
         <v>2.62</v>
@@ -2171,36 +2171,36 @@
         <v>99.74</v>
       </c>
       <c r="U18" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="V18" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="W18" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="X18" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="Y18" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="Z18" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="AA18" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="AB18" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="19" spans="1:28">
       <c r="A19" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B19" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C19" s="2">
         <v>45911</v>
@@ -2215,7 +2215,7 @@
         <v>-85.935445999999999</v>
       </c>
       <c r="G19" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H19" s="6">
         <v>0.3</v>
@@ -2242,7 +2242,7 @@
         <v>3.1</v>
       </c>
       <c r="P19" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q19" s="6">
         <v>2.62</v>
@@ -2257,33 +2257,33 @@
         <v>97.4</v>
       </c>
       <c r="U19" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="V19" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="W19" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="X19" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="Y19" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="Z19" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="AA19" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="20" spans="1:28">
       <c r="A20" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B20" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C20" s="2">
         <v>45911</v>
@@ -2295,78 +2295,78 @@
         <v>-85.971446999999998</v>
       </c>
       <c r="G20" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="K20" s="6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="M20" s="6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="P20" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="Q20" s="6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="R20" s="6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="S20" s="6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="T20" s="6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="U20" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="V20" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="W20" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="X20" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="Y20" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="Z20" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="AA20" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="AB20" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="21" spans="1:28">
       <c r="A21" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B21" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C21" s="2">
         <v>45911</v>
@@ -2378,70 +2378,70 @@
         <v>-85.958196000000001</v>
       </c>
       <c r="G21" t="s">
+        <v>41</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J21" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="K21" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="L21" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="M21" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="N21" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="O21" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="P21" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q21" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="R21" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="S21" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="T21" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="U21" t="s">
+        <v>44</v>
+      </c>
+      <c r="V21" t="s">
+        <v>44</v>
+      </c>
+      <c r="W21" t="s">
+        <v>44</v>
+      </c>
+      <c r="X21" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>44</v>
+      </c>
+      <c r="AB21" t="s">
         <v>45</v>
-      </c>
-      <c r="H21" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="I21" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="J21" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="K21" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="L21" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="M21" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="N21" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="O21" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="P21" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q21" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="R21" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="S21" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="T21" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="U21" t="s">
-        <v>48</v>
-      </c>
-      <c r="V21" t="s">
-        <v>48</v>
-      </c>
-      <c r="W21" t="s">
-        <v>48</v>
-      </c>
-      <c r="X21" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y21" t="s">
-        <v>48</v>
-      </c>
-      <c r="Z21" t="s">
-        <v>48</v>
-      </c>
-      <c r="AA21" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB21" t="s">
-        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Warning: There are less than four response values in stratum "mst_a", the simple random sampling variance estimator for an infinite population was used to calculate variance of the total estimate.
Action: The simple random sampling variance estimator for an infinite population was used.
</commit_message>
<xml_diff>
--- a/survey_wqdata/SR_Data_editsv1.xlsx
+++ b/survey_wqdata/SR_Data_editsv1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\atweg\Documents\Mike\Nokuse\R_sevensrun\nokuse_seven_runs_survey\survey_wqdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B4359B0-8CAD-48D6-A092-F3E29111E965}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ACB82A7-555B-4307-A0E0-30533A45A422}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{BC263282-6D8F-47C7-8BF3-A88688F790FA}"/>
   </bookViews>
@@ -93,9 +93,6 @@
       </rPr>
       <t>˚C)</t>
     </r>
-  </si>
-  <si>
-    <t>pH (SU)</t>
   </si>
   <si>
     <t>D.O. Sat (%)</t>
@@ -258,6 +255,9 @@
   </si>
   <si>
     <t>mck_d</t>
+  </si>
+  <si>
+    <t>pH</t>
   </si>
 </sst>
 </file>
@@ -699,7 +699,7 @@
         <v>15</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H1" s="5" t="s">
         <v>16</v>
@@ -708,69 +708,69 @@
         <v>17</v>
       </c>
       <c r="J1" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="M1" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="N1" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="L1" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="M1" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="N1" s="5" t="s">
+      <c r="O1" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="P1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="R1" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="S1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="Q1" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="R1" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="S1" s="5" t="s">
+      <c r="T1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="T1" s="5" t="s">
+      <c r="U1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="X1" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="Y1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="Z1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="AA1" s="1" t="s">
-        <v>36</v>
-      </c>
       <c r="AB1" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:28">
       <c r="A2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C2" s="2">
         <v>45909</v>
@@ -785,7 +785,7 @@
         <v>-86.038640000000001</v>
       </c>
       <c r="G2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H2" s="6">
         <v>0.25</v>
@@ -812,7 +812,7 @@
         <v>1.63</v>
       </c>
       <c r="P2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Q2" s="6">
         <v>1.37</v>
@@ -827,42 +827,42 @@
         <v>99.48</v>
       </c>
       <c r="U2" t="s">
+        <v>36</v>
+      </c>
+      <c r="V2" t="s">
+        <v>36</v>
+      </c>
+      <c r="W2" t="s">
+        <v>38</v>
+      </c>
+      <c r="X2" t="s">
         <v>37</v>
       </c>
-      <c r="V2" t="s">
-        <v>37</v>
-      </c>
-      <c r="W2" t="s">
-        <v>39</v>
-      </c>
-      <c r="X2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="Z2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="AA2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="AB2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:28">
       <c r="A3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C3" s="2">
         <v>45909</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E3">
         <v>30.574836999999999</v>
@@ -871,7 +871,7 @@
         <v>-86.028282000000004</v>
       </c>
       <c r="G3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H3" s="6">
         <v>0.38</v>
@@ -898,7 +898,7 @@
         <v>2.56</v>
       </c>
       <c r="P3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Q3" s="6">
         <v>2.69</v>
@@ -913,33 +913,33 @@
         <v>95.84</v>
       </c>
       <c r="U3" t="s">
+        <v>36</v>
+      </c>
+      <c r="V3" t="s">
+        <v>36</v>
+      </c>
+      <c r="W3" t="s">
+        <v>38</v>
+      </c>
+      <c r="X3" t="s">
         <v>37</v>
       </c>
-      <c r="V3" t="s">
-        <v>37</v>
-      </c>
-      <c r="W3" t="s">
-        <v>39</v>
-      </c>
-      <c r="X3" t="s">
-        <v>38</v>
-      </c>
       <c r="Y3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="Z3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="AA3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:28">
       <c r="A4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C4" s="2">
         <v>45909</v>
@@ -954,7 +954,7 @@
         <v>-86.016197000000005</v>
       </c>
       <c r="G4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H4" s="6">
         <v>0.4</v>
@@ -981,7 +981,7 @@
         <v>2.14</v>
       </c>
       <c r="P4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Q4" s="6">
         <v>4.83</v>
@@ -996,36 +996,36 @@
         <v>99.48</v>
       </c>
       <c r="U4" t="s">
+        <v>36</v>
+      </c>
+      <c r="V4" t="s">
+        <v>36</v>
+      </c>
+      <c r="W4" t="s">
+        <v>38</v>
+      </c>
+      <c r="X4" t="s">
         <v>37</v>
       </c>
-      <c r="V4" t="s">
-        <v>37</v>
-      </c>
-      <c r="W4" t="s">
-        <v>39</v>
-      </c>
-      <c r="X4" t="s">
-        <v>38</v>
-      </c>
       <c r="Y4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="Z4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="AA4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="AB4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:28">
       <c r="A5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C5" s="2">
         <v>45912</v>
@@ -1040,7 +1040,7 @@
         <v>-85.978043</v>
       </c>
       <c r="G5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H5" s="6">
         <v>0.32</v>
@@ -1067,7 +1067,7 @@
         <v>2.5099999999999998</v>
       </c>
       <c r="P5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Q5" s="6">
         <v>6.45</v>
@@ -1082,39 +1082,39 @@
         <v>84.92</v>
       </c>
       <c r="U5" t="s">
+        <v>36</v>
+      </c>
+      <c r="V5" t="s">
+        <v>36</v>
+      </c>
+      <c r="W5" t="s">
+        <v>38</v>
+      </c>
+      <c r="X5" t="s">
         <v>37</v>
       </c>
-      <c r="V5" t="s">
-        <v>37</v>
-      </c>
-      <c r="W5" t="s">
-        <v>39</v>
-      </c>
-      <c r="X5" t="s">
-        <v>38</v>
-      </c>
       <c r="Y5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="Z5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="AA5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:28">
       <c r="A6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C6" s="2">
         <v>45911</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E6">
         <v>30.556989999999999</v>
@@ -1123,7 +1123,7 @@
         <v>-85.963539999999995</v>
       </c>
       <c r="G6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H6" s="6">
         <v>0.32</v>
@@ -1150,7 +1150,7 @@
         <v>3.71</v>
       </c>
       <c r="P6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Q6" s="6">
         <v>5.13</v>
@@ -1165,33 +1165,33 @@
         <v>96.1</v>
       </c>
       <c r="U6" t="s">
+        <v>36</v>
+      </c>
+      <c r="V6" t="s">
+        <v>36</v>
+      </c>
+      <c r="W6" t="s">
+        <v>38</v>
+      </c>
+      <c r="X6" t="s">
         <v>37</v>
       </c>
-      <c r="V6" t="s">
-        <v>37</v>
-      </c>
-      <c r="W6" t="s">
-        <v>39</v>
-      </c>
-      <c r="X6" t="s">
-        <v>38</v>
-      </c>
       <c r="Y6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="Z6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="AA6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:28">
       <c r="A7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C7" s="2">
         <v>45911</v>
@@ -1206,7 +1206,7 @@
         <v>-85.962569000000002</v>
       </c>
       <c r="G7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H7" s="6">
         <v>0.43</v>
@@ -1233,7 +1233,7 @@
         <v>2.33</v>
       </c>
       <c r="P7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Q7" s="6">
         <v>4.83</v>
@@ -1248,33 +1248,33 @@
         <v>92.72</v>
       </c>
       <c r="U7" t="s">
+        <v>36</v>
+      </c>
+      <c r="V7" t="s">
+        <v>36</v>
+      </c>
+      <c r="W7" t="s">
+        <v>38</v>
+      </c>
+      <c r="X7" t="s">
         <v>37</v>
       </c>
-      <c r="V7" t="s">
-        <v>37</v>
-      </c>
-      <c r="W7" t="s">
-        <v>39</v>
-      </c>
-      <c r="X7" t="s">
-        <v>38</v>
-      </c>
       <c r="Y7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="Z7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="AA7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:28">
       <c r="A8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C8" s="2">
         <v>45910</v>
@@ -1289,7 +1289,7 @@
         <v>-85.979294999999993</v>
       </c>
       <c r="G8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H8" s="6">
         <v>0.32</v>
@@ -1316,7 +1316,7 @@
         <v>1.44</v>
       </c>
       <c r="P8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Q8" s="6">
         <v>1.65</v>
@@ -1331,33 +1331,33 @@
         <v>97.92</v>
       </c>
       <c r="U8" t="s">
+        <v>36</v>
+      </c>
+      <c r="V8" t="s">
+        <v>36</v>
+      </c>
+      <c r="W8" t="s">
+        <v>38</v>
+      </c>
+      <c r="X8" t="s">
         <v>37</v>
       </c>
-      <c r="V8" t="s">
-        <v>37</v>
-      </c>
-      <c r="W8" t="s">
-        <v>39</v>
-      </c>
-      <c r="X8" t="s">
-        <v>38</v>
-      </c>
       <c r="Y8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="Z8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="AA8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:28">
       <c r="A9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C9" s="2">
         <v>45910</v>
@@ -1372,7 +1372,7 @@
         <v>-85.980097000000001</v>
       </c>
       <c r="G9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H9" s="6">
         <v>0.25</v>
@@ -1399,7 +1399,7 @@
         <v>1.74</v>
       </c>
       <c r="P9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Q9" s="6">
         <v>1.0900000000000001</v>
@@ -1414,33 +1414,33 @@
         <v>100</v>
       </c>
       <c r="U9" t="s">
+        <v>36</v>
+      </c>
+      <c r="V9" t="s">
+        <v>36</v>
+      </c>
+      <c r="W9" t="s">
+        <v>38</v>
+      </c>
+      <c r="X9" t="s">
         <v>37</v>
       </c>
-      <c r="V9" t="s">
-        <v>37</v>
-      </c>
-      <c r="W9" t="s">
-        <v>39</v>
-      </c>
-      <c r="X9" t="s">
-        <v>38</v>
-      </c>
       <c r="Y9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="Z9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="AA9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:28">
       <c r="A10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C10" s="2">
         <v>45910</v>
@@ -1455,7 +1455,7 @@
         <v>-85.979523</v>
       </c>
       <c r="G10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H10" s="6">
         <v>0.25</v>
@@ -1482,7 +1482,7 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="P10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Q10" s="6">
         <v>2.82</v>
@@ -1497,42 +1497,42 @@
         <v>98.18</v>
       </c>
       <c r="U10" t="s">
+        <v>36</v>
+      </c>
+      <c r="V10" t="s">
+        <v>36</v>
+      </c>
+      <c r="W10" t="s">
+        <v>38</v>
+      </c>
+      <c r="X10" t="s">
         <v>37</v>
       </c>
-      <c r="V10" t="s">
-        <v>37</v>
-      </c>
-      <c r="W10" t="s">
-        <v>39</v>
-      </c>
-      <c r="X10" t="s">
-        <v>38</v>
-      </c>
       <c r="Y10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="Z10" t="s">
+        <v>50</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>36</v>
+      </c>
+      <c r="AB10" t="s">
         <v>51</v>
-      </c>
-      <c r="AA10" t="s">
-        <v>37</v>
-      </c>
-      <c r="AB10" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:28">
       <c r="A11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C11" s="2">
         <v>45910</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E11">
         <v>30.567005999999999</v>
@@ -1542,7 +1542,7 @@
         <v>-85.979297000000003</v>
       </c>
       <c r="G11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H11" s="6">
         <v>0.34</v>
@@ -1569,7 +1569,7 @@
         <v>3.08</v>
       </c>
       <c r="P11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Q11" s="6">
         <v>2.11</v>
@@ -1584,28 +1584,28 @@
         <v>98.44</v>
       </c>
       <c r="U11" t="s">
+        <v>36</v>
+      </c>
+      <c r="V11" t="s">
+        <v>36</v>
+      </c>
+      <c r="W11" t="s">
+        <v>38</v>
+      </c>
+      <c r="X11" t="s">
         <v>37</v>
       </c>
-      <c r="V11" t="s">
-        <v>37</v>
-      </c>
-      <c r="W11" t="s">
-        <v>39</v>
-      </c>
-      <c r="X11" t="s">
-        <v>38</v>
-      </c>
       <c r="Y11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="Z11" t="s">
+        <v>50</v>
+      </c>
+      <c r="AA11" t="s">
+        <v>36</v>
+      </c>
+      <c r="AB11" t="s">
         <v>51</v>
-      </c>
-      <c r="AA11" t="s">
-        <v>37</v>
-      </c>
-      <c r="AB11" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:28">
@@ -1613,7 +1613,7 @@
         <v>1</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C12" s="2">
         <v>45910</v>
@@ -1628,7 +1628,7 @@
         <v>-85.964935999999994</v>
       </c>
       <c r="G12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H12" s="6">
         <v>0.23</v>
@@ -1655,7 +1655,7 @@
         <v>2</v>
       </c>
       <c r="P12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Q12" s="6">
         <v>1.4</v>
@@ -1670,25 +1670,25 @@
         <v>99.22</v>
       </c>
       <c r="U12" t="s">
+        <v>36</v>
+      </c>
+      <c r="V12" t="s">
+        <v>36</v>
+      </c>
+      <c r="W12" t="s">
+        <v>38</v>
+      </c>
+      <c r="X12" t="s">
         <v>37</v>
       </c>
-      <c r="V12" t="s">
-        <v>37</v>
-      </c>
-      <c r="W12" t="s">
-        <v>39</v>
-      </c>
-      <c r="X12" t="s">
-        <v>38</v>
-      </c>
       <c r="Y12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="Z12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="AA12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:28">
@@ -1696,7 +1696,7 @@
         <v>2</v>
       </c>
       <c r="B13" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C13" s="2">
         <v>45910</v>
@@ -1711,7 +1711,7 @@
         <v>-85.966836999999998</v>
       </c>
       <c r="G13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H13" s="6">
         <v>0.31</v>
@@ -1738,7 +1738,7 @@
         <v>2.48</v>
       </c>
       <c r="P13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Q13" s="6">
         <v>2.74</v>
@@ -1753,25 +1753,25 @@
         <v>99.48</v>
       </c>
       <c r="U13" t="s">
+        <v>36</v>
+      </c>
+      <c r="V13" t="s">
+        <v>36</v>
+      </c>
+      <c r="W13" t="s">
+        <v>38</v>
+      </c>
+      <c r="X13" t="s">
         <v>37</v>
       </c>
-      <c r="V13" t="s">
-        <v>37</v>
-      </c>
-      <c r="W13" t="s">
-        <v>39</v>
-      </c>
-      <c r="X13" t="s">
-        <v>38</v>
-      </c>
       <c r="Y13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="Z13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="AA13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:28">
@@ -1779,7 +1779,7 @@
         <v>3</v>
       </c>
       <c r="B14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C14" s="2">
         <v>45911</v>
@@ -1794,7 +1794,7 @@
         <v>-85.966802999999999</v>
       </c>
       <c r="G14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H14" s="6">
         <v>0.3</v>
@@ -1821,7 +1821,7 @@
         <v>1.85</v>
       </c>
       <c r="P14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Q14" s="6">
         <v>2.62</v>
@@ -1836,25 +1836,25 @@
         <v>97.66</v>
       </c>
       <c r="U14" t="s">
+        <v>36</v>
+      </c>
+      <c r="V14" t="s">
+        <v>36</v>
+      </c>
+      <c r="W14" t="s">
+        <v>38</v>
+      </c>
+      <c r="X14" t="s">
         <v>37</v>
       </c>
-      <c r="V14" t="s">
-        <v>37</v>
-      </c>
-      <c r="W14" t="s">
-        <v>39</v>
-      </c>
-      <c r="X14" t="s">
-        <v>38</v>
-      </c>
       <c r="Y14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="Z14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="AA14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="15" spans="1:28">
@@ -1862,7 +1862,7 @@
         <v>4</v>
       </c>
       <c r="B15" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C15" s="2">
         <v>45912</v>
@@ -1874,70 +1874,70 @@
         <v>-85.984607999999994</v>
       </c>
       <c r="G15" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H15" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="K15" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="L15" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="M15" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="N15" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="O15" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="P15" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q15" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="R15" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="S15" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="T15" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="U15" t="s">
+        <v>43</v>
+      </c>
+      <c r="V15" t="s">
+        <v>43</v>
+      </c>
+      <c r="W15" t="s">
+        <v>43</v>
+      </c>
+      <c r="X15" t="s">
+        <v>43</v>
+      </c>
+      <c r="Y15" t="s">
+        <v>43</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>43</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>43</v>
+      </c>
+      <c r="AB15" t="s">
         <v>44</v>
-      </c>
-      <c r="I15" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="J15" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="K15" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="L15" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M15" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="N15" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="O15" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="P15" t="s">
-        <v>44</v>
-      </c>
-      <c r="Q15" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="R15" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="S15" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="T15" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="U15" t="s">
-        <v>44</v>
-      </c>
-      <c r="V15" t="s">
-        <v>44</v>
-      </c>
-      <c r="W15" t="s">
-        <v>44</v>
-      </c>
-      <c r="X15" t="s">
-        <v>44</v>
-      </c>
-      <c r="Y15" t="s">
-        <v>44</v>
-      </c>
-      <c r="Z15" t="s">
-        <v>44</v>
-      </c>
-      <c r="AA15" t="s">
-        <v>44</v>
-      </c>
-      <c r="AB15" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:28">
@@ -1945,7 +1945,7 @@
         <v>5</v>
       </c>
       <c r="B16" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C16" s="2">
         <v>45912</v>
@@ -1960,7 +1960,7 @@
         <v>-85.981594000000001</v>
       </c>
       <c r="G16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H16" s="6">
         <v>0.22</v>
@@ -1987,7 +1987,7 @@
         <v>3.51</v>
       </c>
       <c r="P16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Q16" s="6">
         <v>2.72</v>
@@ -2002,25 +2002,25 @@
         <v>98.18</v>
       </c>
       <c r="U16" t="s">
+        <v>36</v>
+      </c>
+      <c r="V16" t="s">
+        <v>36</v>
+      </c>
+      <c r="W16" t="s">
+        <v>38</v>
+      </c>
+      <c r="X16" t="s">
         <v>37</v>
       </c>
-      <c r="V16" t="s">
-        <v>37</v>
-      </c>
-      <c r="W16" t="s">
-        <v>39</v>
-      </c>
-      <c r="X16" t="s">
-        <v>38</v>
-      </c>
       <c r="Y16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="Z16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="AA16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17" spans="1:28">
@@ -2028,7 +2028,7 @@
         <v>6</v>
       </c>
       <c r="B17" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C17" s="2">
         <v>45911</v>
@@ -2043,70 +2043,70 @@
         <v>-85.919370000000001</v>
       </c>
       <c r="G17" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L17" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="M17" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="N17" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="O17" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="P17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="Q17" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="R17" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="S17" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="T17" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="U17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="V17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="W17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="X17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="Y17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="Z17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="AA17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="AB17" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:28">
@@ -2114,7 +2114,7 @@
         <v>7</v>
       </c>
       <c r="B18" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C18" s="2">
         <v>45909</v>
@@ -2129,7 +2129,7 @@
         <v>-85.999088</v>
       </c>
       <c r="G18" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H18" s="6">
         <v>0.36</v>
@@ -2156,7 +2156,7 @@
         <v>2.82</v>
       </c>
       <c r="P18" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Q18" s="6">
         <v>2.62</v>
@@ -2171,28 +2171,28 @@
         <v>99.74</v>
       </c>
       <c r="U18" t="s">
+        <v>36</v>
+      </c>
+      <c r="V18" t="s">
+        <v>36</v>
+      </c>
+      <c r="W18" t="s">
+        <v>38</v>
+      </c>
+      <c r="X18" t="s">
         <v>37</v>
       </c>
-      <c r="V18" t="s">
-        <v>37</v>
-      </c>
-      <c r="W18" t="s">
-        <v>39</v>
-      </c>
-      <c r="X18" t="s">
-        <v>38</v>
-      </c>
       <c r="Y18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="Z18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="AA18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="AB18" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="19" spans="1:28">
@@ -2200,7 +2200,7 @@
         <v>8</v>
       </c>
       <c r="B19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C19" s="2">
         <v>45911</v>
@@ -2215,7 +2215,7 @@
         <v>-85.935445999999999</v>
       </c>
       <c r="G19" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H19" s="6">
         <v>0.3</v>
@@ -2242,7 +2242,7 @@
         <v>3.1</v>
       </c>
       <c r="P19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Q19" s="6">
         <v>2.62</v>
@@ -2257,25 +2257,25 @@
         <v>97.4</v>
       </c>
       <c r="U19" t="s">
+        <v>36</v>
+      </c>
+      <c r="V19" t="s">
+        <v>36</v>
+      </c>
+      <c r="W19" t="s">
+        <v>38</v>
+      </c>
+      <c r="X19" t="s">
         <v>37</v>
       </c>
-      <c r="V19" t="s">
-        <v>37</v>
-      </c>
-      <c r="W19" t="s">
-        <v>39</v>
-      </c>
-      <c r="X19" t="s">
-        <v>38</v>
-      </c>
       <c r="Y19" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="Z19" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="AA19" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:28">
@@ -2283,7 +2283,7 @@
         <v>9</v>
       </c>
       <c r="B20" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C20" s="2">
         <v>45911</v>
@@ -2295,70 +2295,70 @@
         <v>-85.971446999999998</v>
       </c>
       <c r="G20" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="K20" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="M20" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="P20" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="Q20" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="R20" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="S20" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="T20" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="U20" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="V20" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="W20" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="X20" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="Y20" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="Z20" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="AA20" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="AB20" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="21" spans="1:28">
@@ -2366,7 +2366,7 @@
         <v>10</v>
       </c>
       <c r="B21" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C21" s="2">
         <v>45911</v>
@@ -2378,70 +2378,70 @@
         <v>-85.958196000000001</v>
       </c>
       <c r="G21" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H21" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="J21" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="K21" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="L21" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="M21" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="N21" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="O21" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="P21" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q21" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="R21" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="S21" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="T21" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="U21" t="s">
+        <v>43</v>
+      </c>
+      <c r="V21" t="s">
+        <v>43</v>
+      </c>
+      <c r="W21" t="s">
+        <v>43</v>
+      </c>
+      <c r="X21" t="s">
+        <v>43</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>43</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>43</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>43</v>
+      </c>
+      <c r="AB21" t="s">
         <v>44</v>
-      </c>
-      <c r="I21" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="J21" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="K21" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="L21" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M21" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="N21" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="O21" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="P21" t="s">
-        <v>44</v>
-      </c>
-      <c r="Q21" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="R21" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="S21" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="T21" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="U21" t="s">
-        <v>44</v>
-      </c>
-      <c r="V21" t="s">
-        <v>44</v>
-      </c>
-      <c r="W21" t="s">
-        <v>44</v>
-      </c>
-      <c r="X21" t="s">
-        <v>44</v>
-      </c>
-      <c r="Y21" t="s">
-        <v>44</v>
-      </c>
-      <c r="Z21" t="s">
-        <v>44</v>
-      </c>
-      <c r="AA21" t="s">
-        <v>44</v>
-      </c>
-      <c r="AB21" t="s">
-        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>